<commit_message>
Add tracking error, information ratio and table formatting updates
</commit_message>
<xml_diff>
--- a/data/dados.xlsx
+++ b/data/dados.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos_Python\kpis_carteira\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos_Python\kpis_carteira\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4179498C-A189-401B-A6A7-A59F4C28E8A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C76D5E5-E1A7-4510-9E44-2BD46208D958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{F37E63D7-3E0E-4B08-A6CB-257A3D200768}"/>
   </bookViews>
@@ -57,10 +57,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="5">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="[$-416]mmmm\-yy;@"/>
+    <numFmt numFmtId="166" formatCode="0.000%"/>
+    <numFmt numFmtId="169" formatCode="_-* #,##0.00000_-;\-* #,##0.00000_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="170" formatCode="_-* #,##0.00000_-;\-* #,##0.00000_-;_-* &quot;-&quot;?????_-;_-@_-"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -70,6 +74,13 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -109,10 +120,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -129,12 +142,23 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentagem" xfId="2" builtinId="5"/>
+    <cellStyle name="Vírgula" xfId="1" builtinId="3"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -466,13 +490,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC365494-2012-4511-855E-1F07D943F801}">
-  <dimension ref="A1:E182"/>
+  <dimension ref="A1:G188"/>
   <sheetFormatPr defaultColWidth="17.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="16384" width="17.85546875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -489,11 +513,11 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>40544</v>
       </c>
-      <c r="B2" s="6">
+      <c r="B2" s="5">
         <v>-1.3531206601987367E-2</v>
       </c>
       <c r="C2" s="2">
@@ -503,8 +527,10 @@
         <v>98.646879339801259</v>
       </c>
       <c r="E2" s="2"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F2" s="8"/>
+      <c r="G2" s="9"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>40575</v>
       </c>
@@ -518,8 +544,10 @@
         <v>99.890595737423283</v>
       </c>
       <c r="E3" s="2"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F3" s="8"/>
+      <c r="G3" s="9"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>40603</v>
       </c>
@@ -533,8 +561,10 @@
         <v>102.99458334289706</v>
       </c>
       <c r="E4" s="2"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F4" s="8"/>
+      <c r="G4" s="9"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>40634</v>
       </c>
@@ -548,8 +578,10 @@
         <v>100.77954247338506</v>
       </c>
       <c r="E5" s="2"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F5" s="8"/>
+      <c r="G5" s="9"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>40694</v>
       </c>
@@ -563,8 +595,10 @@
         <v>99.550088128453197</v>
       </c>
       <c r="E6" s="2"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F6" s="8"/>
+      <c r="G6" s="9"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>40695</v>
       </c>
@@ -578,8 +612,10 @@
         <v>99.202418381909268</v>
       </c>
       <c r="E7" s="2"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F7" s="8"/>
+      <c r="G7" s="9"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>40725</v>
       </c>
@@ -593,8 +629,10 @@
         <v>96.56375796533267</v>
       </c>
       <c r="E8" s="2"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F8" s="8"/>
+      <c r="G8" s="9"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>40756</v>
       </c>
@@ -608,8 +646,10 @@
         <v>94.45362622586677</v>
       </c>
       <c r="E9" s="2"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F9" s="8"/>
+      <c r="G9" s="9"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>40787</v>
       </c>
@@ -623,8 +663,10 @@
         <v>93.703738049624391</v>
       </c>
       <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F10" s="8"/>
+      <c r="G10" s="9"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>40817</v>
       </c>
@@ -638,8 +680,10 @@
         <v>97.479384695396575</v>
       </c>
       <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F11" s="8"/>
+      <c r="G11" s="9"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <v>40848</v>
       </c>
@@ -653,8 +697,10 @@
         <v>97.474266958941186</v>
       </c>
       <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F12" s="8"/>
+      <c r="G12" s="9"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
         <v>40878</v>
       </c>
@@ -670,8 +716,10 @@
       <c r="E13" s="5">
         <v>-1.7923161610526983E-2</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F13" s="8"/>
+      <c r="G13" s="9"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
         <v>40909</v>
       </c>
@@ -687,8 +735,10 @@
       <c r="E14" s="5">
         <v>4.2680529871660822E-2</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F14" s="8"/>
+      <c r="G14" s="9"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>40940</v>
       </c>
@@ -704,8 +754,10 @@
       <c r="E15" s="5">
         <v>5.1583263061345308E-2</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F15" s="8"/>
+      <c r="G15" s="9"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
         <v>40969</v>
       </c>
@@ -721,8 +773,10 @@
       <c r="E16" s="5">
         <v>4.9748059092589836E-2</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F16" s="8"/>
+      <c r="G16" s="9"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>41000</v>
       </c>
@@ -738,8 +792,10 @@
       <c r="E17" s="5">
         <v>3.1757051311789075E-2</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F17" s="8"/>
+      <c r="G17" s="9"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
         <v>41030</v>
       </c>
@@ -755,8 +811,10 @@
       <c r="E18" s="5">
         <v>1.6086174445466339E-2</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F18" s="8"/>
+      <c r="G18" s="9"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="4">
         <v>41061</v>
       </c>
@@ -772,8 +830,10 @@
       <c r="E19" s="5">
         <v>1.5231411810038731E-2</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F19" s="8"/>
+      <c r="G19" s="9"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="4">
         <v>41091</v>
       </c>
@@ -789,8 +849,10 @@
       <c r="E20" s="5">
         <v>3.3173460654560616E-2</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F20" s="8"/>
+      <c r="G20" s="9"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4">
         <v>41122</v>
       </c>
@@ -806,8 +868,10 @@
       <c r="E21" s="5">
         <v>2.947791716538406E-2</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F21" s="8"/>
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <v>41153</v>
       </c>
@@ -823,8 +887,10 @@
       <c r="E22" s="5">
         <v>3.8660481438419492E-2</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F22" s="8"/>
+      <c r="G22" s="9"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
         <v>41183</v>
       </c>
@@ -840,8 +906,10 @@
       <c r="E23" s="5">
         <v>3.9538309397675109E-2</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F23" s="8"/>
+      <c r="G23" s="9"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="4">
         <v>41214</v>
       </c>
@@ -857,8 +925,10 @@
       <c r="E24" s="5">
         <v>5.2350344854978692E-2</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F24" s="8"/>
+      <c r="G24" s="9"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="4">
         <v>41244</v>
       </c>
@@ -874,8 +944,10 @@
       <c r="E25" s="5">
         <v>7.5138362555396965E-2</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F25" s="8"/>
+      <c r="G25" s="9"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
         <v>41275</v>
       </c>
@@ -891,8 +963,10 @@
       <c r="E26" s="5">
         <v>1.0449080250694021E-2</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F26" s="8"/>
+      <c r="G26" s="9"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="4">
         <v>41306</v>
       </c>
@@ -908,8 +982,10 @@
       <c r="E27" s="5">
         <v>-1.3512249110932961E-3</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F27" s="8"/>
+      <c r="G27" s="9"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="4">
         <v>41334</v>
       </c>
@@ -925,8 +1001,10 @@
       <c r="E28" s="5">
         <v>-1.0364991256216149E-2</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F28" s="8"/>
+      <c r="G28" s="9"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="4">
         <v>41365</v>
       </c>
@@ -942,8 +1020,10 @@
       <c r="E29" s="5">
         <v>-4.6253138439178443E-3</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F29" s="8"/>
+      <c r="G29" s="9"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="4">
         <v>41395</v>
       </c>
@@ -959,8 +1039,10 @@
       <c r="E30" s="5">
         <v>-2.5416578623861374E-3</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F30" s="8"/>
+      <c r="G30" s="9"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="4">
         <v>41426</v>
       </c>
@@ -976,8 +1058,10 @@
       <c r="E31" s="5">
         <v>-4.2262507104389946E-2</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F31" s="8"/>
+      <c r="G31" s="9"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="4">
         <v>41456</v>
       </c>
@@ -993,8 +1077,10 @@
       <c r="E32" s="5">
         <v>-3.3408774495763627E-2</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F32" s="8"/>
+      <c r="G32" s="9"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="4">
         <v>41487</v>
       </c>
@@ -1010,8 +1096,10 @@
       <c r="E33" s="5">
         <v>-2.8985933797872399E-2</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F33" s="8"/>
+      <c r="G33" s="9"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="4">
         <v>41518</v>
       </c>
@@ -1027,8 +1115,10 @@
       <c r="E34" s="5">
         <v>-3.9758222812691368E-4</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F34" s="8"/>
+      <c r="G34" s="9"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="4">
         <v>41548</v>
       </c>
@@ -1044,8 +1134,10 @@
       <c r="E35" s="5">
         <v>2.0912975847892756E-2</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F35" s="8"/>
+      <c r="G35" s="9"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="4">
         <v>41579</v>
       </c>
@@ -1061,8 +1153,10 @@
       <c r="E36" s="5">
         <v>1.5381130957244249E-2</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F36" s="8"/>
+      <c r="G36" s="9"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="4">
         <v>41609</v>
       </c>
@@ -1078,8 +1172,10 @@
       <c r="E37" s="5">
         <v>4.7460454778291972E-3</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F37" s="8"/>
+      <c r="G37" s="9"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="4">
         <v>41640</v>
       </c>
@@ -1095,8 +1191,10 @@
       <c r="E38" s="5">
         <v>-3.2485194993333133E-2</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F38" s="8"/>
+      <c r="G38" s="9"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="4">
         <v>41671</v>
       </c>
@@ -1112,8 +1210,10 @@
       <c r="E39" s="5">
         <v>-2.0836049034944293E-2</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F39" s="8"/>
+      <c r="G39" s="9"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="4">
         <v>41699</v>
       </c>
@@ -1129,8 +1229,10 @@
       <c r="E40" s="5">
         <v>5.4536786242698199E-3</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F40" s="8"/>
+      <c r="G40" s="9"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="4">
         <v>41730</v>
       </c>
@@ -1146,8 +1248,10 @@
       <c r="E41" s="5">
         <v>2.3269287630692803E-2</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F41" s="8"/>
+      <c r="G41" s="9"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="4">
         <v>41760</v>
       </c>
@@ -1163,8 +1267,10 @@
       <c r="E42" s="5">
         <v>2.8956225141189451E-2</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F42" s="8"/>
+      <c r="G42" s="9"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="4">
         <v>41791</v>
       </c>
@@ -1180,8 +1286,10 @@
       <c r="E43" s="5">
         <v>4.7820198644879408E-2</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F43" s="8"/>
+      <c r="G43" s="9"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="4">
         <v>41821</v>
       </c>
@@ -1197,8 +1305,10 @@
       <c r="E44" s="5">
         <v>8.1125899145522373E-2</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F44" s="8"/>
+      <c r="G44" s="9"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="4">
         <v>41852</v>
       </c>
@@ -1214,8 +1324,10 @@
       <c r="E45" s="5">
         <v>0.13630989959034912</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F45" s="8"/>
+      <c r="G45" s="9"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="4">
         <v>41883</v>
       </c>
@@ -1231,8 +1343,10 @@
       <c r="E46" s="5">
         <v>7.3251273690771557E-2</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F46" s="8"/>
+      <c r="G46" s="9"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="4">
         <v>41913</v>
       </c>
@@ -1248,8 +1362,10 @@
       <c r="E47" s="5">
         <v>9.6936149249241321E-2</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F47" s="8"/>
+      <c r="G47" s="9"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="4">
         <v>41944</v>
       </c>
@@ -1265,8 +1381,10 @@
       <c r="E48" s="5">
         <v>0.12118845374530585</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F48" s="8"/>
+      <c r="G48" s="9"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="4">
         <v>41974</v>
       </c>
@@ -1282,8 +1400,10 @@
       <c r="E49" s="5">
         <v>7.5009177567250784E-2</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F49" s="8"/>
+      <c r="G49" s="9"/>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="4">
         <v>42005</v>
       </c>
@@ -1299,8 +1419,10 @@
       <c r="E50" s="5">
         <v>-9.4550639303174755E-3</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F50" s="8"/>
+      <c r="G50" s="9"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="4">
         <v>42036</v>
       </c>
@@ -1316,8 +1438,10 @@
       <c r="E51" s="5">
         <v>2.2133129558204123E-2</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F51" s="8"/>
+      <c r="G51" s="9"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="4">
         <v>42064</v>
       </c>
@@ -1333,8 +1457,10 @@
       <c r="E52" s="5">
         <v>2.2008363301832423E-2</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F52" s="8"/>
+      <c r="G52" s="9"/>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="4">
         <v>42095</v>
       </c>
@@ -1350,8 +1476,10 @@
       <c r="E53" s="5">
         <v>6.8574910684546575E-2</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F53" s="8"/>
+      <c r="G53" s="9"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="4">
         <v>42125</v>
       </c>
@@ -1367,8 +1495,10 @@
       <c r="E54" s="5">
         <v>3.7117419870957402E-2</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F54" s="8"/>
+      <c r="G54" s="9"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="4">
         <v>42156</v>
       </c>
@@ -1384,8 +1514,10 @@
       <c r="E55" s="5">
         <v>4.2479890397072229E-2</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F55" s="8"/>
+      <c r="G55" s="9"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="4">
         <v>42186</v>
       </c>
@@ -1401,8 +1533,10 @@
       <c r="E56" s="5">
         <v>3.4617298783850448E-2</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F56" s="8"/>
+      <c r="G56" s="9"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="4">
         <v>42217</v>
       </c>
@@ -1418,8 +1552,10 @@
       <c r="E57" s="5">
         <v>7.9952280268380527E-4</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F57" s="8"/>
+      <c r="G57" s="9"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="4">
         <v>42248</v>
       </c>
@@ -1435,8 +1571,10 @@
       <c r="E58" s="5">
         <v>-3.6908443462515539E-3</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F58" s="8"/>
+      <c r="G58" s="9"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="4">
         <v>42278</v>
       </c>
@@ -1452,8 +1590,10 @@
       <c r="E59" s="5">
         <v>1.4507986544038731E-2</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F59" s="8"/>
+      <c r="G59" s="9"/>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="4">
         <v>42309</v>
       </c>
@@ -1469,8 +1609,10 @@
       <c r="E60" s="5">
         <v>2.9210423602220814E-2</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F60" s="8"/>
+      <c r="G60" s="9"/>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="4">
         <v>42339</v>
       </c>
@@ -1486,8 +1628,10 @@
       <c r="E61" s="5">
         <v>3.5449274396618824E-2</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F61" s="8"/>
+      <c r="G61" s="9"/>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="4">
         <v>42370</v>
       </c>
@@ -1503,8 +1647,10 @@
       <c r="E62" s="5">
         <v>-5.0470073180941544E-4</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F62" s="8"/>
+      <c r="G62" s="9"/>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="4">
         <v>42401</v>
       </c>
@@ -1520,8 +1666,10 @@
       <c r="E63" s="5">
         <v>1.7352805686356776E-2</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F63" s="8"/>
+      <c r="G63" s="9"/>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="4">
         <v>42430</v>
       </c>
@@ -1537,8 +1685,10 @@
       <c r="E64" s="5">
         <v>7.1613256131360936E-2</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F64" s="8"/>
+      <c r="G64" s="9"/>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="4">
         <v>42461</v>
       </c>
@@ -1554,8 +1704,10 @@
       <c r="E65" s="5">
         <v>9.3807728108073585E-2</v>
       </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F65" s="8"/>
+      <c r="G65" s="9"/>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="4">
         <v>42491</v>
       </c>
@@ -1571,8 +1723,10 @@
       <c r="E66" s="5">
         <v>8.4928776522052774E-2</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F66" s="8"/>
+      <c r="G66" s="9"/>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="4">
         <v>42522</v>
       </c>
@@ -1588,8 +1742,10 @@
       <c r="E67" s="5">
         <v>9.3267858050357644E-2</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F67" s="8"/>
+      <c r="G67" s="9"/>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="4">
         <v>42552</v>
       </c>
@@ -1605,8 +1761,10 @@
       <c r="E68" s="5">
         <v>0.13111036280401467</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F68" s="8"/>
+      <c r="G68" s="9"/>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="4">
         <v>42583</v>
       </c>
@@ -1622,8 +1780,10 @@
       <c r="E69" s="5">
         <v>0.14756258525009947</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F69" s="8"/>
+      <c r="G69" s="9"/>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="4">
         <v>42614</v>
       </c>
@@ -1639,8 +1799,10 @@
       <c r="E70" s="5">
         <v>0.15741242302350411</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F70" s="8"/>
+      <c r="G70" s="9"/>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="4">
         <v>42644</v>
       </c>
@@ -1656,8 +1818,10 @@
       <c r="E71" s="5">
         <v>0.19811457076983108</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F71" s="8"/>
+      <c r="G71" s="9"/>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="4">
         <v>42675</v>
       </c>
@@ -1673,8 +1837,10 @@
       <c r="E72" s="5">
         <v>0.19096752496394154</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F72" s="8"/>
+      <c r="G72" s="9"/>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="4">
         <v>42705</v>
       </c>
@@ -1690,8 +1856,10 @@
       <c r="E73" s="5">
         <v>0.19075190194631686</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F73" s="8"/>
+      <c r="G73" s="9"/>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="4">
         <v>42736</v>
       </c>
@@ -1707,8 +1875,10 @@
       <c r="E74" s="5">
         <v>2.5633923135516934E-2</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F74" s="8"/>
+      <c r="G74" s="9"/>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="4">
         <v>42767</v>
       </c>
@@ -1724,8 +1894,10 @@
       <c r="E75" s="5">
         <v>5.7233977016424742E-2</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F75" s="8"/>
+      <c r="G75" s="9"/>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="4">
         <v>42795</v>
       </c>
@@ -1741,8 +1913,10 @@
       <c r="E76" s="5">
         <v>4.9346343496134537E-2</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F76" s="8"/>
+      <c r="G76" s="9"/>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="4">
         <v>42826</v>
       </c>
@@ -1758,8 +1932,10 @@
       <c r="E77" s="5">
         <v>5.1208188908685726E-2</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F77" s="8"/>
+      <c r="G77" s="9"/>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="4">
         <v>42856</v>
       </c>
@@ -1775,8 +1951,10 @@
       <c r="E78" s="5">
         <v>2.8053248720935287E-2</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F78" s="8"/>
+      <c r="G78" s="9"/>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="4">
         <v>42887</v>
       </c>
@@ -1792,8 +1970,10 @@
       <c r="E79" s="5">
         <v>4.5867470336370397E-2</v>
       </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F79" s="8"/>
+      <c r="G79" s="9"/>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="4">
         <v>42917</v>
       </c>
@@ -1809,8 +1989,10 @@
       <c r="E80" s="5">
         <v>7.6687581073999089E-2</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F80" s="8"/>
+      <c r="G80" s="9"/>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="4">
         <v>42948</v>
       </c>
@@ -1826,8 +2008,10 @@
       <c r="E81" s="5">
         <v>0.10886556970553474</v>
       </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F81" s="8"/>
+      <c r="G81" s="9"/>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="4">
         <v>42979</v>
       </c>
@@ -1843,8 +2027,10 @@
       <c r="E82" s="5">
         <v>0.14636799572474124</v>
       </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F82" s="8"/>
+      <c r="G82" s="9"/>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="4">
         <v>43009</v>
       </c>
@@ -1860,8 +2046,10 @@
       <c r="E83" s="5">
         <v>0.14823626692688019</v>
       </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F83" s="8"/>
+      <c r="G83" s="9"/>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="4">
         <v>43040</v>
       </c>
@@ -1877,8 +2065,10 @@
       <c r="E84" s="5">
         <v>0.134657742484664</v>
       </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F84" s="8"/>
+      <c r="G84" s="9"/>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="4">
         <v>43070</v>
       </c>
@@ -1894,8 +2084,10 @@
       <c r="E85" s="5">
         <v>0.15724353488325904</v>
       </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F85" s="8"/>
+      <c r="G85" s="9"/>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="4">
         <v>43101</v>
       </c>
@@ -1911,8 +2103,10 @@
       <c r="E86" s="5">
         <v>6.9065174710739363E-2</v>
       </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F86" s="8"/>
+      <c r="G86" s="9"/>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="4">
         <v>43132</v>
       </c>
@@ -1928,8 +2122,10 @@
       <c r="E87" s="5">
         <v>6.8351274859855371E-2</v>
       </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F87" s="8"/>
+      <c r="G87" s="9"/>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="4">
         <v>43160</v>
       </c>
@@ -1945,8 +2141,10 @@
       <c r="E88" s="5">
         <v>7.2834109036970629E-2</v>
       </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F88" s="8"/>
+      <c r="G88" s="9"/>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="4">
         <v>43191</v>
       </c>
@@ -1962,8 +2160,10 @@
       <c r="E89" s="5">
         <v>8.2514581901377504E-2</v>
       </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F89" s="8"/>
+      <c r="G89" s="9"/>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="4">
         <v>43221</v>
       </c>
@@ -1979,8 +2179,10 @@
       <c r="E90" s="5">
         <v>2.9231514415205995E-2</v>
       </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F90" s="8"/>
+      <c r="G90" s="9"/>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="4">
         <v>43252</v>
       </c>
@@ -1996,8 +2198,10 @@
       <c r="E91" s="5">
         <v>7.8451051933783322E-3</v>
       </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F91" s="8"/>
+      <c r="G91" s="9"/>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="4">
         <v>43282</v>
       </c>
@@ -2013,8 +2217,10 @@
       <c r="E92" s="5">
         <v>5.3524535453640221E-2</v>
       </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F92" s="8"/>
+      <c r="G92" s="9"/>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="4">
         <v>43313</v>
       </c>
@@ -2030,8 +2236,10 @@
       <c r="E93" s="5">
         <v>4.8647588728380153E-2</v>
       </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F93" s="8"/>
+      <c r="G93" s="9"/>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="4">
         <v>43344</v>
       </c>
@@ -2047,8 +2255,10 @@
       <c r="E94" s="5">
         <v>5.9569921522242275E-2</v>
       </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F94" s="8"/>
+      <c r="G94" s="9"/>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="4">
         <v>43374</v>
       </c>
@@ -2064,8 +2274,10 @@
       <c r="E95" s="5">
         <v>0.115376120705311</v>
       </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F95" s="8"/>
+      <c r="G95" s="9"/>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="4">
         <v>43405</v>
       </c>
@@ -2081,8 +2293,10 @@
       <c r="E96" s="5">
         <v>0.14701486880928294</v>
       </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F96" s="8"/>
+      <c r="G96" s="9"/>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="4">
         <v>43435</v>
       </c>
@@ -2098,8 +2312,10 @@
       <c r="E97" s="5">
         <v>0.14006532857375786</v>
       </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F97" s="8"/>
+      <c r="G97" s="9"/>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="4">
         <v>43466</v>
       </c>
@@ -2115,8 +2331,10 @@
       <c r="E98" s="5">
         <v>5.8449715234484723E-2</v>
       </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F98" s="8"/>
+      <c r="G98" s="9"/>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="4">
         <v>43497</v>
       </c>
@@ -2132,8 +2350,10 @@
       <c r="E99" s="5">
         <v>5.6446973929201949E-2</v>
       </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F99" s="8"/>
+      <c r="G99" s="9"/>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="4">
         <v>43525</v>
       </c>
@@ -2149,8 +2369,10 @@
       <c r="E100" s="5">
         <v>6.7780022212966973E-2</v>
       </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F100" s="8"/>
+      <c r="G100" s="9"/>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="4">
         <v>43556</v>
       </c>
@@ -2166,8 +2388,10 @@
       <c r="E101" s="5">
         <v>7.9242639852410868E-2</v>
       </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F101" s="8"/>
+      <c r="G101" s="9"/>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="4">
         <v>43586</v>
       </c>
@@ -2183,8 +2407,10 @@
       <c r="E102" s="5">
         <v>9.6546932778789341E-2</v>
       </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F102" s="8"/>
+      <c r="G102" s="9"/>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" s="4">
         <v>43617</v>
       </c>
@@ -2200,8 +2426,10 @@
       <c r="E103" s="5">
         <v>0.14782741988889514</v>
       </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F103" s="8"/>
+      <c r="G103" s="9"/>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="4">
         <v>43647</v>
       </c>
@@ -2217,8 +2445,10 @@
       <c r="E104" s="5">
         <v>0.15492335404332436</v>
       </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F104" s="8"/>
+      <c r="G104" s="9"/>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="4">
         <v>43678</v>
       </c>
@@ -2234,8 +2464,10 @@
       <c r="E105" s="5">
         <v>0.14972623375554983</v>
       </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F105" s="8"/>
+      <c r="G105" s="9"/>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="4">
         <v>43709</v>
       </c>
@@ -2251,8 +2483,10 @@
       <c r="E106" s="5">
         <v>0.18295511511740625</v>
       </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F106" s="8"/>
+      <c r="G106" s="9"/>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="4">
         <v>43739</v>
       </c>
@@ -2268,8 +2502,10 @@
       <c r="E107" s="5">
         <v>0.21918227399823964</v>
       </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F107" s="8"/>
+      <c r="G107" s="9"/>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="4">
         <v>43770</v>
       </c>
@@ -2285,8 +2521,10 @@
       <c r="E108" s="5">
         <v>0.22619274773085185</v>
       </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F108" s="8"/>
+      <c r="G108" s="9"/>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" s="4">
         <v>43800</v>
       </c>
@@ -2302,8 +2540,10 @@
       <c r="E109" s="5">
         <v>0.25726036989209522</v>
       </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F109" s="8"/>
+      <c r="G109" s="9"/>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="4">
         <v>43831</v>
       </c>
@@ -2319,8 +2559,10 @@
       <c r="E110" s="5">
         <v>5.524508751617585E-3</v>
       </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F110" s="8"/>
+      <c r="G110" s="9"/>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="4">
         <v>43862</v>
       </c>
@@ -2336,8 +2578,10 @@
       <c r="E111" s="5">
         <v>-1.9926769825587942E-2</v>
       </c>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F111" s="8"/>
+      <c r="G111" s="9"/>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" s="4">
         <v>43891</v>
       </c>
@@ -2353,8 +2597,10 @@
       <c r="E112" s="5">
         <v>-0.13590023661143658</v>
       </c>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F112" s="8"/>
+      <c r="G112" s="9"/>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" s="4">
         <v>43922</v>
       </c>
@@ -2370,8 +2616,10 @@
       <c r="E113" s="5">
         <v>-9.8705292162029057E-2</v>
       </c>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F113" s="8"/>
+      <c r="G113" s="9"/>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" s="4">
         <v>43952</v>
       </c>
@@ -2387,8 +2635,10 @@
       <c r="E114" s="5">
         <v>-7.7207518515168605E-2</v>
       </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F114" s="8"/>
+      <c r="G114" s="9"/>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" s="4">
         <v>43983</v>
       </c>
@@ -2404,8 +2654,10 @@
       <c r="E115" s="5">
         <v>-4.7038542129020922E-2</v>
       </c>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F115" s="8"/>
+      <c r="G115" s="9"/>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" s="4">
         <v>44013</v>
       </c>
@@ -2421,8 +2673,10 @@
       <c r="E116" s="5">
         <v>3.7331987145823309E-3</v>
       </c>
-    </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F116" s="8"/>
+      <c r="G116" s="9"/>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" s="4">
         <v>44044</v>
       </c>
@@ -2438,8 +2692,10 @@
       <c r="E117" s="5">
         <v>2.9867278414772658E-2</v>
       </c>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F117" s="8"/>
+      <c r="G117" s="9"/>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118" s="4">
         <v>44075</v>
       </c>
@@ -2455,8 +2711,10 @@
       <c r="E118" s="5">
         <v>-3.4170183998971648E-4</v>
       </c>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F118" s="8"/>
+      <c r="G118" s="9"/>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" s="4">
         <v>44105</v>
       </c>
@@ -2472,8 +2730,10 @@
       <c r="E119" s="5">
         <v>-6.2516434973379775E-3</v>
       </c>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F119" s="8"/>
+      <c r="G119" s="9"/>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" s="4">
         <v>44136</v>
       </c>
@@ -2489,8 +2749,10 @@
       <c r="E120" s="5">
         <v>4.1930041352205683E-2</v>
       </c>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F120" s="8"/>
+      <c r="G120" s="9"/>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" s="4">
         <v>44166</v>
       </c>
@@ -2506,8 +2768,10 @@
       <c r="E121" s="5">
         <v>8.1567968705213545E-2</v>
       </c>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F121" s="8"/>
+      <c r="G121" s="9"/>
+    </row>
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" s="4">
         <v>44197</v>
       </c>
@@ -2523,8 +2787,10 @@
       <c r="E122" s="5">
         <v>1.7501001444384157E-2</v>
       </c>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F122" s="8"/>
+      <c r="G122" s="9"/>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123" s="4">
         <v>44228</v>
       </c>
@@ -2540,8 +2806,10 @@
       <c r="E123" s="5">
         <v>1.7051291043106209E-2</v>
       </c>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F123" s="8"/>
+      <c r="G123" s="9"/>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" s="4">
         <v>44256</v>
       </c>
@@ -2557,8 +2825,10 @@
       <c r="E124" s="5">
         <v>4.3571856127858188E-2</v>
       </c>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F124" s="8"/>
+      <c r="G124" s="9"/>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" s="4">
         <v>44287</v>
       </c>
@@ -2574,8 +2844,10 @@
       <c r="E125" s="5">
         <v>7.7299985019803286E-2</v>
       </c>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F125" s="8"/>
+      <c r="G125" s="9"/>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126" s="4">
         <v>44317</v>
       </c>
@@ -2591,8 +2863,10 @@
       <c r="E126" s="5">
         <v>8.063649325346911E-2</v>
       </c>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F126" s="8"/>
+      <c r="G126" s="9"/>
+    </row>
+    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127" s="4">
         <v>44348</v>
       </c>
@@ -2608,8 +2882,10 @@
       <c r="E127" s="5">
         <v>8.3328145852292979E-2</v>
       </c>
-    </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F127" s="8"/>
+      <c r="G127" s="9"/>
+    </row>
+    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128" s="4">
         <v>44378</v>
       </c>
@@ -2625,8 +2901,10 @@
       <c r="E128" s="5">
         <v>9.6204523701672651E-2</v>
       </c>
-    </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F128" s="8"/>
+      <c r="G128" s="9"/>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129" s="4">
         <v>44409</v>
       </c>
@@ -2642,8 +2920,10 @@
       <c r="E129" s="5">
         <v>9.9557201390430006E-2</v>
       </c>
-    </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F129" s="8"/>
+      <c r="G129" s="9"/>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A130" s="4">
         <v>44440</v>
       </c>
@@ -2659,8 +2939,10 @@
       <c r="E130" s="5">
         <v>9.2145672763783049E-2</v>
       </c>
-    </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F130" s="8"/>
+      <c r="G130" s="9"/>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131" s="4">
         <v>44470</v>
       </c>
@@ -2676,8 +2958,10 @@
       <c r="E131" s="5">
         <v>0.14753938613162498</v>
       </c>
-    </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F131" s="8"/>
+      <c r="G131" s="9"/>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132" s="4">
         <v>44501</v>
       </c>
@@ -2693,8 +2977,10 @@
       <c r="E132" s="5">
         <v>0.12306127828726843</v>
       </c>
-    </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F132" s="8"/>
+      <c r="G132" s="9"/>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A133" s="4">
         <v>44531</v>
       </c>
@@ -2710,8 +2996,10 @@
       <c r="E133" s="5">
         <v>0.15807671108996302</v>
       </c>
-    </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F133" s="8"/>
+      <c r="G133" s="9"/>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134" s="4">
         <v>44562</v>
       </c>
@@ -2727,8 +3015,10 @@
       <c r="E134" s="5">
         <v>-6.3689308112705678E-2</v>
       </c>
-    </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F134" s="8"/>
+      <c r="G134" s="9"/>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A135" s="4">
         <v>44593</v>
       </c>
@@ -2744,8 +3034,10 @@
       <c r="E135" s="5">
         <v>-9.2743341907106758E-2</v>
       </c>
-    </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F135" s="8"/>
+      <c r="G135" s="9"/>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136" s="4">
         <v>44621</v>
       </c>
@@ -2761,8 +3053,10 @@
       <c r="E136" s="5">
         <v>-0.11115124418525302</v>
       </c>
-    </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F136" s="8"/>
+      <c r="G136" s="9"/>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137" s="4">
         <v>44652</v>
       </c>
@@ -2778,8 +3072,10 @@
       <c r="E137" s="5">
         <v>-0.1503924506550528</v>
       </c>
-    </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F137" s="8"/>
+      <c r="G137" s="9"/>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138" s="4">
         <v>44682</v>
       </c>
@@ -2795,8 +3091,10 @@
       <c r="E138" s="5">
         <v>-0.18364219332019416</v>
       </c>
-    </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F138" s="8"/>
+      <c r="G138" s="9"/>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139" s="4">
         <v>44713</v>
       </c>
@@ -2812,8 +3110,10 @@
       <c r="E139" s="5">
         <v>-0.19050371116209919</v>
       </c>
-    </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F139" s="8"/>
+      <c r="G139" s="9"/>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140" s="4">
         <v>44743</v>
       </c>
@@ -2829,8 +3129,10 @@
       <c r="E140" s="5">
         <v>-0.14913850585460042</v>
       </c>
-    </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F140" s="8"/>
+      <c r="G140" s="9"/>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141" s="4">
         <v>44774</v>
       </c>
@@ -2846,8 +3148,10 @@
       <c r="E141" s="5">
         <v>-0.16749227140096123</v>
       </c>
-    </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F141" s="8"/>
+      <c r="G141" s="9"/>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142" s="4">
         <v>44805</v>
       </c>
@@ -2863,8 +3167,10 @@
       <c r="E142" s="5">
         <v>-0.22341540241088542</v>
       </c>
-    </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F142" s="8"/>
+      <c r="G142" s="9"/>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143" s="4">
         <v>44835</v>
       </c>
@@ -2880,8 +3186,10 @@
       <c r="E143" s="5">
         <v>-0.2082534500393376</v>
       </c>
-    </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F143" s="8"/>
+      <c r="G143" s="9"/>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144" s="4">
         <v>44866</v>
       </c>
@@ -2897,8 +3205,10 @@
       <c r="E144" s="5">
         <v>-0.15859424635086283</v>
       </c>
-    </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F144" s="8"/>
+      <c r="G144" s="9"/>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A145" s="4">
         <v>44896</v>
       </c>
@@ -2914,8 +3224,10 @@
       <c r="E145" s="5">
         <v>-0.17000742952282966</v>
       </c>
-    </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F145" s="8"/>
+      <c r="G145" s="9"/>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A146" s="4">
         <v>44927</v>
       </c>
@@ -2931,8 +3243,10 @@
       <c r="E146" s="5">
         <v>4.1617975729686174E-2</v>
       </c>
-    </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F146" s="8"/>
+      <c r="G146" s="9"/>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A147" s="4">
         <v>44958</v>
       </c>
@@ -2948,8 +3262,10 @@
       <c r="E147" s="5">
         <v>3.64664335833631E-2</v>
       </c>
-    </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F147" s="8"/>
+      <c r="G147" s="9"/>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148" s="4">
         <v>44986</v>
       </c>
@@ -2965,8 +3281,10 @@
       <c r="E148" s="5">
         <v>2.0544325411329556E-2</v>
       </c>
-    </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F148" s="8"/>
+      <c r="G148" s="9"/>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A149" s="4">
         <v>45017</v>
       </c>
@@ -2982,8 +3300,10 @@
       <c r="E149" s="5">
         <v>2.3930390073236163E-2</v>
       </c>
-    </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F149" s="8"/>
+      <c r="G149" s="9"/>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150" s="4">
         <v>45047</v>
       </c>
@@ -2999,8 +3319,10 @@
       <c r="E150" s="5">
         <v>2.3726410274193421E-2</v>
       </c>
-    </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F150" s="8"/>
+      <c r="G150" s="9"/>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A151" s="4">
         <v>45078</v>
       </c>
@@ -3016,8 +3338,10 @@
       <c r="E151" s="5">
         <v>4.7618145826552993E-2</v>
       </c>
-    </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F151" s="8"/>
+      <c r="G151" s="9"/>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A152" s="4">
         <v>45108</v>
       </c>
@@ -3033,8 +3357,10 @@
       <c r="E152" s="5">
         <v>8.6550358473693967E-2</v>
       </c>
-    </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F152" s="8"/>
+      <c r="G152" s="9"/>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A153" s="4">
         <v>45139</v>
       </c>
@@ -3050,8 +3376,10 @@
       <c r="E153" s="5">
         <v>8.6941818525568593E-2</v>
       </c>
-    </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F153" s="8"/>
+      <c r="G153" s="9"/>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A154" s="4">
         <v>45170</v>
       </c>
@@ -3067,8 +3395,10 @@
       <c r="E154" s="5">
         <v>5.9205926007695142E-2</v>
       </c>
-    </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F154" s="8"/>
+      <c r="G154" s="9"/>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A155" s="4">
         <v>45200</v>
       </c>
@@ -3084,8 +3414,10 @@
       <c r="E155" s="5">
         <v>1.5963298657311276E-2</v>
       </c>
-    </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F155" s="8"/>
+      <c r="G155" s="9"/>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A156" s="4">
         <v>45231</v>
       </c>
@@ -3101,8 +3433,10 @@
       <c r="E156" s="5">
         <v>8.8038153378697359E-2</v>
       </c>
-    </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F156" s="8"/>
+      <c r="G156" s="9"/>
+    </row>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A157" s="4">
         <v>45261</v>
       </c>
@@ -3118,8 +3452,10 @@
       <c r="E157" s="5">
         <v>0.14722581785348132</v>
       </c>
-    </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F157" s="8"/>
+      <c r="G157" s="9"/>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A158" s="4">
         <v>45292</v>
       </c>
@@ -3135,8 +3471,10 @@
       <c r="E158" s="5">
         <v>1.4136673240136011E-2</v>
       </c>
-    </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F158" s="8"/>
+      <c r="G158" s="9"/>
+    </row>
+    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A159" s="4">
         <v>45323</v>
       </c>
@@ -3152,8 +3490,10 @@
       <c r="E159" s="5">
         <v>4.5579316826681371E-2</v>
       </c>
-    </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F159" s="8"/>
+      <c r="G159" s="9"/>
+    </row>
+    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A160" s="4">
         <v>45352</v>
       </c>
@@ -3169,8 +3509,10 @@
       <c r="E160" s="5">
         <v>6.8349293054297489E-2</v>
       </c>
-    </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F160" s="8"/>
+      <c r="G160" s="9"/>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A161" s="4">
         <v>45383</v>
       </c>
@@ -3186,8 +3528,10 @@
       <c r="E161" s="5">
         <v>7.281254964725381E-2</v>
       </c>
-    </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F161" s="8"/>
+      <c r="G161" s="9"/>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A162" s="4">
         <v>45413</v>
       </c>
@@ -3203,8 +3547,10 @@
       <c r="E162" s="5">
         <v>0.11123318379664271</v>
       </c>
-    </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F162" s="8"/>
+      <c r="G162" s="9"/>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A163" s="4">
         <v>45444</v>
       </c>
@@ -3220,8 +3566,10 @@
       <c r="E163" s="5">
         <v>0.20072780943969515</v>
       </c>
-    </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F163" s="8"/>
+      <c r="G163" s="9"/>
+    </row>
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A164" s="4">
         <v>45474</v>
       </c>
@@ -3237,8 +3585,10 @@
       <c r="E164" s="5">
         <v>0.25924950781287959</v>
       </c>
-    </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F164" s="8"/>
+      <c r="G164" s="9"/>
+    </row>
+    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A165" s="4">
         <v>45505</v>
       </c>
@@ -3254,8 +3604,10 @@
       <c r="E165" s="5">
         <v>0.27821998533461501</v>
       </c>
-    </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F165" s="8"/>
+      <c r="G165" s="9"/>
+    </row>
+    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A166" s="4">
         <v>45536</v>
       </c>
@@ -3271,8 +3623,10 @@
       <c r="E166" s="5">
         <v>0.2698518207957854</v>
       </c>
-    </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F166" s="8"/>
+      <c r="G166" s="9"/>
+    </row>
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A167" s="4">
         <v>45566</v>
       </c>
@@ -3288,8 +3642,10 @@
       <c r="E167" s="5">
         <v>0.31722540582655689</v>
       </c>
-    </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F167" s="8"/>
+      <c r="G167" s="9"/>
+    </row>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168" s="4">
         <v>45597</v>
       </c>
@@ -3305,8 +3661,10 @@
       <c r="E168" s="5">
         <v>0.4137287501892033</v>
       </c>
-    </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F168" s="8"/>
+      <c r="G168" s="9"/>
+    </row>
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A169" s="4">
         <v>45627</v>
       </c>
@@ -3322,8 +3680,10 @@
       <c r="E169" s="5">
         <v>0.40956937844071906</v>
       </c>
-    </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F169" s="8"/>
+      <c r="G169" s="9"/>
+    </row>
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A170" s="4">
         <v>45658</v>
       </c>
@@ -3339,8 +3699,10 @@
       <c r="E170" s="5">
         <v>-2.0550296327777606E-2</v>
       </c>
-    </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F170" s="8"/>
+      <c r="G170" s="9"/>
+    </row>
+    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A171" s="4">
         <v>45689</v>
       </c>
@@ -3356,8 +3718,10 @@
       <c r="E171" s="5">
         <v>-2.4816341148991894E-2</v>
       </c>
-    </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F171" s="8"/>
+      <c r="G171" s="9"/>
+    </row>
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A172" s="4">
         <v>45717</v>
       </c>
@@ -3373,8 +3737,10 @@
       <c r="E172" s="5">
         <v>-8.4361377395558268E-2</v>
       </c>
-    </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F172" s="8"/>
+      <c r="G172" s="9"/>
+    </row>
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A173" s="4">
         <v>45748</v>
       </c>
@@ -3390,8 +3756,10 @@
       <c r="E173" s="5">
         <v>-9.1783937400516713E-2</v>
       </c>
-    </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F173" s="8"/>
+      <c r="G173" s="9"/>
+    </row>
+    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A174" s="4">
         <v>45778</v>
       </c>
@@ -3407,8 +3775,10 @@
       <c r="E174" s="5">
         <v>-2.7802956111603883E-2</v>
       </c>
-    </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F174" s="8"/>
+      <c r="G174" s="9"/>
+    </row>
+    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A175" s="4">
         <v>45809</v>
       </c>
@@ -3424,8 +3794,10 @@
       <c r="E175" s="5">
         <v>-2.8087495990421707E-2</v>
       </c>
-    </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F175" s="8"/>
+      <c r="G175" s="9"/>
+    </row>
+    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A176" s="4">
         <v>45839</v>
       </c>
@@ -3441,8 +3813,10 @@
       <c r="E176" s="5">
         <v>1.9039136137490642E-2</v>
       </c>
-    </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F176" s="8"/>
+      <c r="G176" s="9"/>
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A177" s="4">
         <v>45870</v>
       </c>
@@ -3458,8 +3832,10 @@
       <c r="E177" s="5">
         <v>2.2526300959900158E-2</v>
       </c>
-    </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F177" s="8"/>
+      <c r="G177" s="9"/>
+    </row>
+    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A178" s="4">
         <v>45901</v>
       </c>
@@ -3475,8 +3851,10 @@
       <c r="E178" s="5">
         <v>3.4249835386125804E-2</v>
       </c>
-    </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F178" s="8"/>
+      <c r="G178" s="9"/>
+    </row>
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A179" s="4">
         <v>45931</v>
       </c>
@@ -3492,8 +3870,10 @@
       <c r="E179" s="5">
         <v>7.8855262053866504E-2</v>
       </c>
-    </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F179" s="8"/>
+      <c r="G179" s="9"/>
+    </row>
+    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A180" s="4">
         <v>45962</v>
       </c>
@@ -3509,8 +3889,10 @@
       <c r="E180" s="5">
         <v>7.8439970091665145E-2</v>
       </c>
-    </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F180" s="8"/>
+      <c r="G180" s="9"/>
+    </row>
+    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A181" s="4">
         <v>45992</v>
       </c>
@@ -3526,8 +3908,10 @@
       <c r="E181" s="5">
         <v>0.13278122177380203</v>
       </c>
-    </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F181" s="8"/>
+      <c r="G181" s="9"/>
+    </row>
+    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A182" s="4">
         <v>46023</v>
       </c>
@@ -3543,6 +3927,14 @@
       <c r="E182" s="5">
         <v>6.7310504859385833E-3</v>
       </c>
+      <c r="F182" s="8"/>
+      <c r="G182" s="9"/>
+    </row>
+    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G183" s="7"/>
+    </row>
+    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G188" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
feat: update portfolio analytics KPIs and diagnostic reports
</commit_message>
<xml_diff>
--- a/data/dados.xlsx
+++ b/data/dados.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos_Python\kpis_carteira\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C76D5E5-E1A7-4510-9E44-2BD46208D958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C460B1E5-DA74-4817-85C7-D9631430004C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{F37E63D7-3E0E-4B08-A6CB-257A3D200768}"/>
   </bookViews>
@@ -60,9 +60,9 @@
   <numFmts count="5">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="[$-416]mmmm\-yy;@"/>
-    <numFmt numFmtId="166" formatCode="0.000%"/>
-    <numFmt numFmtId="169" formatCode="_-* #,##0.00000_-;\-* #,##0.00000_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="170" formatCode="_-* #,##0.00000_-;\-* #,##0.00000_-;_-* &quot;-&quot;?????_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="0.000%"/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0.00000_-;\-* #,##0.00000_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="167" formatCode="_-* #,##0.00000_-;\-* #,##0.00000_-;_-* &quot;-&quot;?????_-;_-@_-"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -145,13 +145,13 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3931,6 +3931,21 @@
       <c r="G182" s="9"/>
     </row>
     <row r="183" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A183" s="4">
+        <v>46054</v>
+      </c>
+      <c r="B183" s="5">
+        <v>9.514059145745879E-3</v>
+      </c>
+      <c r="C183" s="2">
+        <v>451.41994036251026</v>
+      </c>
+      <c r="D183" s="2">
+        <v>101.63091492441207</v>
+      </c>
+      <c r="E183" s="5">
+        <v>1.6309149244120746E-2</v>
+      </c>
       <c r="G183" s="7"/>
     </row>
     <row r="188" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>